<commit_message>
data: replace bookstore samples with updated marketplace datasets
</commit_message>
<xml_diff>
--- a/sample-data/Don_Hang_POS.xlsx
+++ b/sample-data/Don_Hang_POS.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R38290a49ad854363"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="Rf4e70789ac9749b7"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -330,7 +330,7 @@
         <x:v>9786045200261</x:v>
       </x:c>
       <x:c r="D2" s="12" t="str">
-        <x:v>Vợ Nhặt</x:v>
+        <x:v>Vợ Nhặt (Bản thường)</x:v>
       </x:c>
       <x:c r="E2" s="12" t="n">
         <x:v>1</x:v>
@@ -362,7 +362,7 @@
         <x:v>9786045200476</x:v>
       </x:c>
       <x:c r="D3" s="12" t="str">
-        <x:v>Nghĩ Giàu Làm Giàu</x:v>
+        <x:v>Nghĩ Giàu Làm Giàu (Bản thường)</x:v>
       </x:c>
       <x:c r="E3" s="12" t="n">
         <x:v>1</x:v>
@@ -391,10 +391,10 @@
         <x:v>POS-2025-003</x:v>
       </x:c>
       <x:c r="C4" s="12" t="str">
-        <x:v>9786045200179</x:v>
+        <x:v>9786041200179</x:v>
       </x:c>
       <x:c r="D4" s="12" t="str">
-        <x:v>Cha Giàu Cha Nghèo</x:v>
+        <x:v>Cha Giàu Cha Nghèo (Bản thường)</x:v>
       </x:c>
       <x:c r="E4" s="12" t="n">
         <x:v>1</x:v>
@@ -426,7 +426,7 @@
         <x:v>9786045200445</x:v>
       </x:c>
       <x:c r="D5" s="12" t="str">
-        <x:v>Muôn Kiếp Nhân Sinh</x:v>
+        <x:v>Muôn Kiếp Nhân Sinh (Bản thường)</x:v>
       </x:c>
       <x:c r="E5" s="12" t="n">
         <x:v>1</x:v>
@@ -458,7 +458,7 @@
         <x:v>9786045200278</x:v>
       </x:c>
       <x:c r="D6" s="12" t="str">
-        <x:v>Bố Già</x:v>
+        <x:v>Bố Già (Bản thường)</x:v>
       </x:c>
       <x:c r="E6" s="12" t="n">
         <x:v>1</x:v>
@@ -487,10 +487,10 @@
         <x:v>POS-2025-006</x:v>
       </x:c>
       <x:c r="C7" s="12" t="str">
-        <x:v>9786043950106</x:v>
+        <x:v>9786042001063</x:v>
       </x:c>
       <x:c r="D7" s="12" t="str">
-        <x:v>Dế Mèn Phiêu Lưu Ký</x:v>
+        <x:v>Dế Mèn Phiêu Lưu Ký (Bản thường)</x:v>
       </x:c>
       <x:c r="E7" s="12" t="n">
         <x:v>1</x:v>
@@ -519,10 +519,10 @@
         <x:v>POS-2025-007</x:v>
       </x:c>
       <x:c r="C8" s="12" t="str">
-        <x:v>9786043950212</x:v>
+        <x:v>9786042002121</x:v>
       </x:c>
       <x:c r="D8" s="12" t="str">
-        <x:v>One Piece - Tập 100</x:v>
+        <x:v>One Piece - Tập 100 (Bản thường)</x:v>
       </x:c>
       <x:c r="E8" s="12" t="n">
         <x:v>1</x:v>
@@ -551,10 +551,10 @@
         <x:v>POS-2025-008</x:v>
       </x:c>
       <x:c r="C9" s="12" t="str">
-        <x:v>9786045200223</x:v>
+        <x:v>9786041200223</x:v>
       </x:c>
       <x:c r="D9" s="12" t="str">
-        <x:v>Chainsaw Man - Tập 1</x:v>
+        <x:v>Chainsaw Man - Tập 1 (Bản thường)</x:v>
       </x:c>
       <x:c r="E9" s="12" t="n">
         <x:v>1</x:v>
@@ -586,7 +586,7 @@
         <x:v>9786043950557</x:v>
       </x:c>
       <x:c r="D10" s="12" t="str">
-        <x:v>Light Novel Liệu Có Sai Lầm Khi Tìm Kiếm Kẻ Thù Trong Hầm Ngục - Tập 1</x:v>
+        <x:v>Liệu Có Sai Lầm Khi Tìm Kiếm Cuộc Gặp Gỡ Định Mệnh Trong Dungeon? - Tập 1 (Bản thường)</x:v>
       </x:c>
       <x:c r="E10" s="12" t="n">
         <x:v>1</x:v>
@@ -615,10 +615,10 @@
         <x:v>POS-2025-010</x:v>
       </x:c>
       <x:c r="C11" s="12" t="str">
-        <x:v>9786045200025</x:v>
+        <x:v>9786041273955</x:v>
       </x:c>
       <x:c r="D11" s="12" t="str">
-        <x:v>Tôi Thấy Hoa Vàng Trên Cỏ Xanh</x:v>
+        <x:v>Tôi Thấy Hoa Vàng Trên Cỏ Xanh (Bản thường)</x:v>
       </x:c>
       <x:c r="E11" s="12" t="n">
         <x:v>2</x:v>
@@ -650,7 +650,7 @@
         <x:v>9786045200438</x:v>
       </x:c>
       <x:c r="D12" s="12" t="str">
-        <x:v>Totto-chan Bên Cửa Sổ</x:v>
+        <x:v>Totto-chan Bên Cửa Sổ (Bản thường)</x:v>
       </x:c>
       <x:c r="E12" s="12" t="n">
         <x:v>1</x:v>
@@ -682,7 +682,7 @@
         <x:v>9786045200506</x:v>
       </x:c>
       <x:c r="D13" s="12" t="str">
-        <x:v>Sapiens Lược Sử Loài Người</x:v>
+        <x:v>Sapiens - Lược Sử Loài Người (Bản thường)</x:v>
       </x:c>
       <x:c r="E13" s="12" t="n">
         <x:v>1</x:v>
@@ -714,7 +714,7 @@
         <x:v>9786045200278</x:v>
       </x:c>
       <x:c r="D14" s="12" t="str">
-        <x:v>Bố Già</x:v>
+        <x:v>Bố Già (Bản thường)</x:v>
       </x:c>
       <x:c r="E14" s="12" t="n">
         <x:v>1</x:v>
@@ -746,7 +746,7 @@
         <x:v>9786045200124</x:v>
       </x:c>
       <x:c r="D15" s="12" t="str">
-        <x:v>Tuổi Trẻ Đáng Giá Bao Nhiêu</x:v>
+        <x:v>Tuổi Trẻ Đáng Giá Bao Nhiêu (Bản thường)</x:v>
       </x:c>
       <x:c r="E15" s="12" t="n">
         <x:v>1</x:v>
@@ -778,7 +778,7 @@
         <x:v>9786045200506</x:v>
       </x:c>
       <x:c r="D16" s="12" t="str">
-        <x:v>Sapiens Lược Sử Loài Người</x:v>
+        <x:v>Sapiens - Lược Sử Loài Người (Bản thường)</x:v>
       </x:c>
       <x:c r="E16" s="12" t="n">
         <x:v>1</x:v>
@@ -810,7 +810,7 @@
         <x:v>9786045200261</x:v>
       </x:c>
       <x:c r="D17" s="12" t="str">
-        <x:v>Vợ Nhặt</x:v>
+        <x:v>Vợ Nhặt (Bản thường)</x:v>
       </x:c>
       <x:c r="E17" s="12" t="n">
         <x:v>1</x:v>
@@ -842,7 +842,7 @@
         <x:v>9786043950458</x:v>
       </x:c>
       <x:c r="D18" s="12" t="str">
-        <x:v>Light Novel Re:Zero - Bắt Đầu Lại Ở Thế Giới Khác - Tập 1</x:v>
+        <x:v>Re:Zero - Bắt Đầu Lại Ở Thế Giới Khác - Tập 1 (Bản thường)</x:v>
       </x:c>
       <x:c r="E18" s="12" t="n">
         <x:v>1</x:v>
@@ -871,10 +871,10 @@
         <x:v>POS-2025-018</x:v>
       </x:c>
       <x:c r="C19" s="12" t="str">
-        <x:v>9786045200285</x:v>
+        <x:v>9786047200285</x:v>
       </x:c>
       <x:c r="D19" s="12" t="str">
-        <x:v>Quốc Gia Khởi Nghiệp</x:v>
+        <x:v>Quốc Gia Khởi Nghiệp (Bản thường)</x:v>
       </x:c>
       <x:c r="E19" s="12" t="n">
         <x:v>1</x:v>
@@ -906,7 +906,7 @@
         <x:v>9786045200124</x:v>
       </x:c>
       <x:c r="D20" s="12" t="str">
-        <x:v>Tuổi Trẻ Đáng Giá Bao Nhiêu</x:v>
+        <x:v>Tuổi Trẻ Đáng Giá Bao Nhiêu (Bản thường)</x:v>
       </x:c>
       <x:c r="E20" s="12" t="n">
         <x:v>1</x:v>
@@ -938,7 +938,7 @@
         <x:v>9786045200537</x:v>
       </x:c>
       <x:c r="D21" s="12" t="str">
-        <x:v>Tắt Đèn</x:v>
+        <x:v>Tắt Đèn (Bản thường)</x:v>
       </x:c>
       <x:c r="E21" s="12" t="n">
         <x:v>1</x:v>
@@ -970,7 +970,7 @@
         <x:v>9786045200407</x:v>
       </x:c>
       <x:c r="D22" s="12" t="str">
-        <x:v>Nhà Giả Kim</x:v>
+        <x:v>Nhà Giả Kim (Bản thường)</x:v>
       </x:c>
       <x:c r="E22" s="12" t="n">
         <x:v>1</x:v>
@@ -1002,7 +1002,7 @@
         <x:v>9786045200506</x:v>
       </x:c>
       <x:c r="D23" s="12" t="str">
-        <x:v>Sapiens Lược Sử Loài Người</x:v>
+        <x:v>Sapiens - Lược Sử Loài Người (Bản thường)</x:v>
       </x:c>
       <x:c r="E23" s="12" t="n">
         <x:v>1</x:v>
@@ -1031,10 +1031,10 @@
         <x:v>POS-2025-023</x:v>
       </x:c>
       <x:c r="C24" s="12" t="str">
-        <x:v>9786045200568</x:v>
+        <x:v>9786047200568</x:v>
       </x:c>
       <x:c r="D24" s="12" t="str">
-        <x:v>Bản Đồ Cảm Xúc</x:v>
+        <x:v>Bản Đồ Cảm Xúc (Bản thường)</x:v>
       </x:c>
       <x:c r="E24" s="12" t="n">
         <x:v>1</x:v>
@@ -1066,7 +1066,7 @@
         <x:v>9786045200353</x:v>
       </x:c>
       <x:c r="D25" s="12" t="str">
-        <x:v>Bài Học Diệu Kỳ Từ Cây Táo</x:v>
+        <x:v>Bài Học Diệu Kỳ Từ Cây Táo (Bản thường)</x:v>
       </x:c>
       <x:c r="E25" s="12" t="n">
         <x:v>2</x:v>
@@ -1098,7 +1098,7 @@
         <x:v>9786045200537</x:v>
       </x:c>
       <x:c r="D26" s="12" t="str">
-        <x:v>Tắt Đèn</x:v>
+        <x:v>Tắt Đèn (Bản thường)</x:v>
       </x:c>
       <x:c r="E26" s="12" t="n">
         <x:v>1</x:v>
@@ -1127,10 +1127,10 @@
         <x:v>POS-2025-026</x:v>
       </x:c>
       <x:c r="C27" s="12" t="str">
-        <x:v>9786043950014</x:v>
+        <x:v>9786049500141</x:v>
       </x:c>
       <x:c r="D27" s="12" t="str">
-        <x:v>Mãi Mãi Tuổi Hai Mươi (Độc quyền - Bìa cứng)</x:v>
+        <x:v>Mãi Mãi Tuổi Hai Mươi (Bản đặc biệt)</x:v>
       </x:c>
       <x:c r="E27" s="12" t="n">
         <x:v>1</x:v>
@@ -1162,7 +1162,7 @@
         <x:v>9786045200049</x:v>
       </x:c>
       <x:c r="D28" s="12" t="str">
-        <x:v>Chiếc Thuyền Ngoài Xa</x:v>
+        <x:v>Chiếc Th thuyền Ngoài Xa (Bản thường)</x:v>
       </x:c>
       <x:c r="E28" s="12" t="n">
         <x:v>1</x:v>
@@ -1191,10 +1191,10 @@
         <x:v>POS-2025-028</x:v>
       </x:c>
       <x:c r="C29" s="12" t="str">
-        <x:v>9786043950014</x:v>
+        <x:v>9786049500141</x:v>
       </x:c>
       <x:c r="D29" s="12" t="str">
-        <x:v>Mãi Mãi Tuổi Hai Mươi (Độc quyền - Bìa cứng)</x:v>
+        <x:v>Mãi Mãi Tuổi Hai Mươi (Bản đặc biệt)</x:v>
       </x:c>
       <x:c r="E29" s="12" t="n">
         <x:v>1</x:v>
@@ -1226,7 +1226,7 @@
         <x:v>9786045200049</x:v>
       </x:c>
       <x:c r="D30" s="12" t="str">
-        <x:v>Chiếc Thuyền Ngoài Xa</x:v>
+        <x:v>Chiếc Th thuyền Ngoài Xa (Bản thường)</x:v>
       </x:c>
       <x:c r="E30" s="12" t="n">
         <x:v>1</x:v>
@@ -1255,10 +1255,10 @@
         <x:v>POS-2025-030</x:v>
       </x:c>
       <x:c r="C31" s="12" t="str">
-        <x:v>9786045200155</x:v>
+        <x:v>9786041200155</x:v>
       </x:c>
       <x:c r="D31" s="12" t="str">
-        <x:v>Mắt Biếc</x:v>
+        <x:v>Mắt Biếc (Bản thường)</x:v>
       </x:c>
       <x:c r="E31" s="12" t="n">
         <x:v>1</x:v>
@@ -1287,7 +1287,7 @@
         <x:v>POS-2025-031</x:v>
       </x:c>
       <x:c r="C32" s="12" t="str">
-        <x:v>9786043950304</x:v>
+        <x:v>9786042003045</x:v>
       </x:c>
       <x:c r="D32" s="12" t="str">
         <x:v>Dragon Ball Super - Tập 1 (Tái bản)</x:v>
@@ -1322,7 +1322,7 @@
         <x:v>9786045200315</x:v>
       </x:c>
       <x:c r="D33" s="12" t="str">
-        <x:v>Điểm Đến Của Cuộc Đời</x:v>
+        <x:v>Điểm Đến Của Cuộc Đời (Bản thường)</x:v>
       </x:c>
       <x:c r="E33" s="12" t="n">
         <x:v>1</x:v>
@@ -1351,10 +1351,10 @@
         <x:v>POS-2025-033</x:v>
       </x:c>
       <x:c r="C34" s="12" t="str">
-        <x:v>9786045200186</x:v>
+        <x:v>9786041200186</x:v>
       </x:c>
       <x:c r="D34" s="12" t="str">
-        <x:v>Cà Phê Cùng Tony</x:v>
+        <x:v>Cà Phê Cùng Tony (Bản thường)</x:v>
       </x:c>
       <x:c r="E34" s="12" t="n">
         <x:v>1</x:v>
@@ -1386,7 +1386,7 @@
         <x:v>9786045200544</x:v>
       </x:c>
       <x:c r="D35" s="12" t="str">
-        <x:v>Rừng Na Uy</x:v>
+        <x:v>Rừng Na Uy (Bản thường)</x:v>
       </x:c>
       <x:c r="E35" s="12" t="n">
         <x:v>1</x:v>
@@ -1418,7 +1418,7 @@
         <x:v>9786045200353</x:v>
       </x:c>
       <x:c r="D36" s="12" t="str">
-        <x:v>Bài Học Diệu Kỳ Từ Cây Táo</x:v>
+        <x:v>Bài Học Diệu Kỳ Từ Cây Táo (Bản thường)</x:v>
       </x:c>
       <x:c r="E36" s="12" t="n">
         <x:v>1</x:v>
@@ -1447,10 +1447,10 @@
         <x:v>POS-2025-036</x:v>
       </x:c>
       <x:c r="C37" s="12" t="str">
-        <x:v>9786043950526</x:v>
+        <x:v>9786042005269</x:v>
       </x:c>
       <x:c r="D37" s="12" t="str">
-        <x:v>Spy x Family - Tập 1</x:v>
+        <x:v>Spy x Family - Tập 1 (Bản thường)</x:v>
       </x:c>
       <x:c r="E37" s="12" t="n">
         <x:v>1</x:v>
@@ -1479,10 +1479,10 @@
         <x:v>POS-2025-037</x:v>
       </x:c>
       <x:c r="C38" s="12" t="str">
-        <x:v>9786043950113</x:v>
+        <x:v>9786042001131</x:v>
       </x:c>
       <x:c r="D38" s="12" t="str">
-        <x:v>Dragon Ball Super - Tập 2</x:v>
+        <x:v>Dragon Ball Super - Tập 2 (Bản thường)</x:v>
       </x:c>
       <x:c r="E38" s="12" t="n">
         <x:v>1</x:v>
@@ -1514,7 +1514,7 @@
         <x:v>9786045200506</x:v>
       </x:c>
       <x:c r="D39" s="12" t="str">
-        <x:v>Sapiens Lược Sử Loài Người</x:v>
+        <x:v>Sapiens - Lược Sử Loài Người (Bản thường)</x:v>
       </x:c>
       <x:c r="E39" s="12" t="n">
         <x:v>1</x:v>
@@ -1543,10 +1543,10 @@
         <x:v>POS-2025-039</x:v>
       </x:c>
       <x:c r="C40" s="12" t="str">
-        <x:v>9786045200339</x:v>
+        <x:v>9786041200339</x:v>
       </x:c>
       <x:c r="D40" s="12" t="str">
-        <x:v>Trên Đường Băng</x:v>
+        <x:v>Trên Đường Băng (Bản thường)</x:v>
       </x:c>
       <x:c r="E40" s="12" t="n">
         <x:v>1</x:v>
@@ -1578,7 +1578,7 @@
         <x:v>9786045200131</x:v>
       </x:c>
       <x:c r="D41" s="12" t="str">
-        <x:v>Hoàng Tử Bé</x:v>
+        <x:v>Hoàng Tử Bé (Bản thường)</x:v>
       </x:c>
       <x:c r="E41" s="12" t="n">
         <x:v>1</x:v>
@@ -1610,7 +1610,7 @@
         <x:v>9786045200360</x:v>
       </x:c>
       <x:c r="D42" s="12" t="str">
-        <x:v>Bước Chậm Lại Giữa Thế Gian Vội Vã</x:v>
+        <x:v>Bước Chậm Lại Giữa Thế Gian Vội Vã (Bản thường)</x:v>
       </x:c>
       <x:c r="E42" s="12" t="n">
         <x:v>1</x:v>
@@ -1639,10 +1639,10 @@
         <x:v>POS-2025-042</x:v>
       </x:c>
       <x:c r="C43" s="12" t="str">
-        <x:v>9786045200346</x:v>
+        <x:v>9786041200346</x:v>
       </x:c>
       <x:c r="D43" s="12" t="str">
-        <x:v>Fire Force - Biệt Đội Lính Cứu Hỏa - Tập 1</x:v>
+        <x:v>Fire Force - Biệt Đội Lính Cứu Hỏa - Tập 1 (Bản thường)</x:v>
       </x:c>
       <x:c r="E43" s="12" t="n">
         <x:v>1</x:v>
@@ -1674,7 +1674,7 @@
         <x:v>9786045200292</x:v>
       </x:c>
       <x:c r="D44" s="12" t="str">
-        <x:v>Light Novel Vì Con Gái Tôi Có Thể Đánh Bại Cả Ma Vương - Tập 1</x:v>
+        <x:v>Vì Con Gái Tôi Có Thể Đánh Bại Cả Ma Vương - Tập 1 (Bản thường)</x:v>
       </x:c>
       <x:c r="E44" s="12" t="n">
         <x:v>1</x:v>
@@ -1706,7 +1706,7 @@
         <x:v>9786045200483</x:v>
       </x:c>
       <x:c r="D45" s="12" t="str">
-        <x:v>Sức Mạnh Của Hiện Tại</x:v>
+        <x:v>Sức Mạnh Của Hiện Tại (Bản thường)</x:v>
       </x:c>
       <x:c r="E45" s="12" t="n">
         <x:v>1</x:v>
@@ -1735,10 +1735,10 @@
         <x:v>POS-2025-045</x:v>
       </x:c>
       <x:c r="C46" s="12" t="str">
-        <x:v>9786045200155</x:v>
+        <x:v>9786041200155</x:v>
       </x:c>
       <x:c r="D46" s="12" t="str">
-        <x:v>Mắt Biếc</x:v>
+        <x:v>Mắt Biếc (Bản thường)</x:v>
       </x:c>
       <x:c r="E46" s="12" t="n">
         <x:v>1</x:v>
@@ -1770,7 +1770,7 @@
         <x:v>9786045200162</x:v>
       </x:c>
       <x:c r="D47" s="12" t="str">
-        <x:v>Hạt Giống Tâm Hồn</x:v>
+        <x:v>Hạt Giống Tâm Hồn (Bản thường)</x:v>
       </x:c>
       <x:c r="E47" s="12" t="n">
         <x:v>1</x:v>
@@ -1799,10 +1799,10 @@
         <x:v>POS-2025-047</x:v>
       </x:c>
       <x:c r="C48" s="12" t="str">
-        <x:v>9786043950526</x:v>
+        <x:v>9786042005269</x:v>
       </x:c>
       <x:c r="D48" s="12" t="str">
-        <x:v>Spy x Family - Tập 1</x:v>
+        <x:v>Spy x Family - Tập 1 (Bản thường)</x:v>
       </x:c>
       <x:c r="E48" s="12" t="n">
         <x:v>1</x:v>
@@ -1831,10 +1831,10 @@
         <x:v>POS-2025-048</x:v>
       </x:c>
       <x:c r="C49" s="12" t="str">
-        <x:v>9786043950113</x:v>
+        <x:v>9786042001131</x:v>
       </x:c>
       <x:c r="D49" s="12" t="str">
-        <x:v>Dragon Ball Super - Tập 2</x:v>
+        <x:v>Dragon Ball Super - Tập 2 (Bản thường)</x:v>
       </x:c>
       <x:c r="E49" s="12" t="n">
         <x:v>1</x:v>
@@ -1863,10 +1863,10 @@
         <x:v>POS-2025-049</x:v>
       </x:c>
       <x:c r="C50" s="12" t="str">
-        <x:v>9786045200223</x:v>
+        <x:v>9786041200223</x:v>
       </x:c>
       <x:c r="D50" s="12" t="str">
-        <x:v>Chainsaw Man - Tập 1</x:v>
+        <x:v>Chainsaw Man - Tập 1 (Bản thường)</x:v>
       </x:c>
       <x:c r="E50" s="12" t="n">
         <x:v>1</x:v>
@@ -1898,7 +1898,7 @@
         <x:v>9786043950090</x:v>
       </x:c>
       <x:c r="D51" s="12" t="str">
-        <x:v>Light Novel Overlord - Tập 1 - Bất Tử Vương</x:v>
+        <x:v>Overlord - Tập 1: Bất Tử Vương (Bản thường)</x:v>
       </x:c>
       <x:c r="E51" s="12" t="n">
         <x:v>1</x:v>
@@ -1927,10 +1927,10 @@
         <x:v>POS-2025-051</x:v>
       </x:c>
       <x:c r="C52" s="12" t="str">
-        <x:v>9786045200148</x:v>
+        <x:v>9786047200148</x:v>
       </x:c>
       <x:c r="D52" s="12" t="str">
-        <x:v>Tâm Lý Học Đám Đông</x:v>
+        <x:v>Tâm Lý Học Đám Đông (Bản thường)</x:v>
       </x:c>
       <x:c r="E52" s="12" t="n">
         <x:v>1</x:v>
@@ -1959,10 +1959,10 @@
         <x:v>POS-2025-052</x:v>
       </x:c>
       <x:c r="C53" s="12" t="str">
-        <x:v>9786045200186</x:v>
+        <x:v>9786041200186</x:v>
       </x:c>
       <x:c r="D53" s="12" t="str">
-        <x:v>Cà Phê Cùng Tony</x:v>
+        <x:v>Cà Phê Cùng Tony (Bản thường)</x:v>
       </x:c>
       <x:c r="E53" s="12" t="n">
         <x:v>1</x:v>
@@ -1994,7 +1994,7 @@
         <x:v>9786045200513</x:v>
       </x:c>
       <x:c r="D54" s="12" t="str">
-        <x:v>Đọc Vị Bất Kỳ Ai</x:v>
+        <x:v>Đọc Vị Bất Kỳ Ai (Bản thường)</x:v>
       </x:c>
       <x:c r="E54" s="12" t="n">
         <x:v>1</x:v>
@@ -2026,7 +2026,7 @@
         <x:v>9786045200513</x:v>
       </x:c>
       <x:c r="D55" s="12" t="str">
-        <x:v>Đọc Vị Bất Kỳ Ai</x:v>
+        <x:v>Đọc Vị Bất Kỳ Ai (Bản thường)</x:v>
       </x:c>
       <x:c r="E55" s="12" t="n">
         <x:v>1</x:v>
@@ -2055,10 +2055,10 @@
         <x:v>POS-2025-055</x:v>
       </x:c>
       <x:c r="C56" s="12" t="str">
-        <x:v>9786045200025</x:v>
+        <x:v>9786041273955</x:v>
       </x:c>
       <x:c r="D56" s="12" t="str">
-        <x:v>Tôi Thấy Hoa Vàng Trên Cỏ Xanh</x:v>
+        <x:v>Tôi Thấy Hoa Vàng Trên Cỏ Xanh (Bản thường)</x:v>
       </x:c>
       <x:c r="E56" s="12" t="n">
         <x:v>1</x:v>
@@ -2090,7 +2090,7 @@
         <x:v>9786043950557</x:v>
       </x:c>
       <x:c r="D57" s="12" t="str">
-        <x:v>Light Novel Liệu Có Sai Lầm Khi Tìm Kiếm Kẻ Thù Trong Hầm Ngục - Tập 1</x:v>
+        <x:v>Liệu Có Sai Lầm Khi Tìm Kiếm Cuộc Gặp Gỡ Định Mệnh Trong Dungeon? - Tập 1 (Bản thường)</x:v>
       </x:c>
       <x:c r="E57" s="12" t="n">
         <x:v>1</x:v>
@@ -2119,10 +2119,10 @@
         <x:v>POS-2025-057</x:v>
       </x:c>
       <x:c r="C58" s="12" t="str">
-        <x:v>9786045200339</x:v>
+        <x:v>9786041200339</x:v>
       </x:c>
       <x:c r="D58" s="12" t="str">
-        <x:v>Trên Đường Băng</x:v>
+        <x:v>Trên Đường Băng (Bản thường)</x:v>
       </x:c>
       <x:c r="E58" s="12" t="n">
         <x:v>1</x:v>
@@ -2151,10 +2151,10 @@
         <x:v>POS-2025-058</x:v>
       </x:c>
       <x:c r="C59" s="12" t="str">
-        <x:v>9786045200285</x:v>
+        <x:v>9786047200285</x:v>
       </x:c>
       <x:c r="D59" s="12" t="str">
-        <x:v>Quốc Gia Khởi Nghiệp</x:v>
+        <x:v>Quốc Gia Khởi Nghiệp (Bản thường)</x:v>
       </x:c>
       <x:c r="E59" s="12" t="n">
         <x:v>1</x:v>
@@ -2183,10 +2183,10 @@
         <x:v>POS-2025-059</x:v>
       </x:c>
       <x:c r="C60" s="12" t="str">
-        <x:v>9786045200186</x:v>
+        <x:v>9786041200186</x:v>
       </x:c>
       <x:c r="D60" s="12" t="str">
-        <x:v>Cà Phê Cùng Tony</x:v>
+        <x:v>Cà Phê Cùng Tony (Bản thường)</x:v>
       </x:c>
       <x:c r="E60" s="12" t="n">
         <x:v>1</x:v>
@@ -2215,10 +2215,10 @@
         <x:v>POS-2025-060</x:v>
       </x:c>
       <x:c r="C61" s="12" t="str">
-        <x:v>9786043950014</x:v>
+        <x:v>9786049500141</x:v>
       </x:c>
       <x:c r="D61" s="12" t="str">
-        <x:v>Mãi Mãi Tuổi Hai Mươi (Độc quyền - Bìa cứng)</x:v>
+        <x:v>Mãi Mãi Tuổi Hai Mươi (Bản đặc biệt)</x:v>
       </x:c>
       <x:c r="E61" s="12" t="n">
         <x:v>1</x:v>
@@ -2247,10 +2247,10 @@
         <x:v>POS-2025-061</x:v>
       </x:c>
       <x:c r="C62" s="12" t="str">
-        <x:v>9786045200568</x:v>
+        <x:v>9786047200568</x:v>
       </x:c>
       <x:c r="D62" s="12" t="str">
-        <x:v>Bản Đồ Cảm Xúc</x:v>
+        <x:v>Bản Đồ Cảm Xúc (Bản thường)</x:v>
       </x:c>
       <x:c r="E62" s="12" t="n">
         <x:v>1</x:v>
@@ -2282,7 +2282,7 @@
         <x:v>9786045200353</x:v>
       </x:c>
       <x:c r="D63" s="12" t="str">
-        <x:v>Bài Học Diệu Kỳ Từ Cây Táo</x:v>
+        <x:v>Bài Học Diệu Kỳ Từ Cây Táo (Bản thường)</x:v>
       </x:c>
       <x:c r="E63" s="12" t="n">
         <x:v>1</x:v>
@@ -2311,10 +2311,10 @@
         <x:v>POS-2025-063</x:v>
       </x:c>
       <x:c r="C64" s="12" t="str">
-        <x:v>9786045200346</x:v>
+        <x:v>9786041200346</x:v>
       </x:c>
       <x:c r="D64" s="12" t="str">
-        <x:v>Fire Force - Biệt Đội Lính Cứu Hỏa - Tập 1</x:v>
+        <x:v>Fire Force - Biệt Đội Lính Cứu Hỏa - Tập 1 (Bản thường)</x:v>
       </x:c>
       <x:c r="E64" s="12" t="n">
         <x:v>2</x:v>
@@ -2346,7 +2346,7 @@
         <x:v>9786043950557</x:v>
       </x:c>
       <x:c r="D65" s="12" t="str">
-        <x:v>Light Novel Liệu Có Sai Lầm Khi Tìm Kiếm Kẻ Thù Trong Hầm Ngục - Tập 1</x:v>
+        <x:v>Liệu Có Sai Lầm Khi Tìm Kiếm Cuộc Gặp Gỡ Định Mệnh Trong Dungeon? - Tập 1 (Bản thường)</x:v>
       </x:c>
       <x:c r="E65" s="12" t="n">
         <x:v>1</x:v>
@@ -2378,7 +2378,7 @@
         <x:v>9786045200032</x:v>
       </x:c>
       <x:c r="D66" s="12" t="str">
-        <x:v>Chuyện Con Mèo Dạy Hải Âu Bay</x:v>
+        <x:v>Chuyện Con Mèo Dạy Hải Âu Bay (Bản thường)</x:v>
       </x:c>
       <x:c r="E66" s="12" t="n">
         <x:v>1</x:v>
@@ -2410,7 +2410,7 @@
         <x:v>9786043950410</x:v>
       </x:c>
       <x:c r="D67" s="12" t="str">
-        <x:v>Light Novel Sword Art Online 001 - Aincrad</x:v>
+        <x:v>Sword Art Online 001 - Aincrad (Bản thường)</x:v>
       </x:c>
       <x:c r="E67" s="12" t="n">
         <x:v>1</x:v>
@@ -2442,7 +2442,7 @@
         <x:v>9786045200445</x:v>
       </x:c>
       <x:c r="D68" s="12" t="str">
-        <x:v>Muôn Kiếp Nhân Sinh</x:v>
+        <x:v>Muôn Kiếp Nhân Sinh (Bản thường)</x:v>
       </x:c>
       <x:c r="E68" s="12" t="n">
         <x:v>1</x:v>
@@ -2474,7 +2474,7 @@
         <x:v>9786045200360</x:v>
       </x:c>
       <x:c r="D69" s="12" t="str">
-        <x:v>Bước Chậm Lại Giữa Thế Gian Vội Vã</x:v>
+        <x:v>Bước Chậm Lại Giữa Thế Gian Vội Vã (Bản thường)</x:v>
       </x:c>
       <x:c r="E69" s="12" t="n">
         <x:v>1</x:v>
@@ -2506,7 +2506,7 @@
         <x:v>9786045200483</x:v>
       </x:c>
       <x:c r="D70" s="12" t="str">
-        <x:v>Sức Mạnh Của Hiện Tại</x:v>
+        <x:v>Sức Mạnh Của Hiện Tại (Bản thường)</x:v>
       </x:c>
       <x:c r="E70" s="12" t="n">
         <x:v>1</x:v>
@@ -2535,10 +2535,10 @@
         <x:v>POS-2025-070</x:v>
       </x:c>
       <x:c r="C71" s="12" t="str">
-        <x:v>9786045200186</x:v>
+        <x:v>9786041200186</x:v>
       </x:c>
       <x:c r="D71" s="12" t="str">
-        <x:v>Cà Phê Cùng Tony</x:v>
+        <x:v>Cà Phê Cùng Tony (Bản thường)</x:v>
       </x:c>
       <x:c r="E71" s="12" t="n">
         <x:v>1</x:v>
@@ -2567,10 +2567,10 @@
         <x:v>POS-2025-071</x:v>
       </x:c>
       <x:c r="C72" s="12" t="str">
-        <x:v>9786043950069</x:v>
+        <x:v>9786042000691</x:v>
       </x:c>
       <x:c r="D72" s="12" t="str">
-        <x:v>Naruto - Tập 1: Uzumaki Naruto</x:v>
+        <x:v>Naruto - Tập 1: Uzumaki Naruto (Bản thường)</x:v>
       </x:c>
       <x:c r="E72" s="12" t="n">
         <x:v>1</x:v>
@@ -2602,7 +2602,7 @@
         <x:v>9786045200131</x:v>
       </x:c>
       <x:c r="D73" s="12" t="str">
-        <x:v>Hoàng Tử Bé</x:v>
+        <x:v>Hoàng Tử Bé (Bản thường)</x:v>
       </x:c>
       <x:c r="E73" s="12" t="n">
         <x:v>1</x:v>
@@ -2631,10 +2631,10 @@
         <x:v>POS-2025-073</x:v>
       </x:c>
       <x:c r="C74" s="12" t="str">
-        <x:v>9786045200087</x:v>
+        <x:v>9786041000870</x:v>
       </x:c>
       <x:c r="D74" s="12" t="str">
-        <x:v>Nhà Lãnh Đạo Không Chức Danh</x:v>
+        <x:v>Nhà Lãnh Đạo Không Chức Danh (Bản thường)</x:v>
       </x:c>
       <x:c r="E74" s="12" t="n">
         <x:v>1</x:v>
@@ -2666,7 +2666,7 @@
         <x:v>9786045200322</x:v>
       </x:c>
       <x:c r="D75" s="12" t="str">
-        <x:v>Khéo Ăn Nói Sẽ Có Được Thiên Hạ</x:v>
+        <x:v>Khéo Ăn Nói Sẽ Có Được Thiên Hạ (Bản thường)</x:v>
       </x:c>
       <x:c r="E75" s="12" t="n">
         <x:v>1</x:v>
@@ -2698,7 +2698,7 @@
         <x:v>9786045200315</x:v>
       </x:c>
       <x:c r="D76" s="12" t="str">
-        <x:v>Điểm Đến Của Cuộc Đời</x:v>
+        <x:v>Điểm Đến Của Cuộc Đời (Bản thường)</x:v>
       </x:c>
       <x:c r="E76" s="12" t="n">
         <x:v>2</x:v>
@@ -2730,7 +2730,7 @@
         <x:v>9786045200209</x:v>
       </x:c>
       <x:c r="D77" s="12" t="str">
-        <x:v>Kafka Bên Bờ Biển</x:v>
+        <x:v>Kafka Bên Bờ Biển (Bản thường)</x:v>
       </x:c>
       <x:c r="E77" s="12" t="n">
         <x:v>1</x:v>
@@ -2762,7 +2762,7 @@
         <x:v>9786045200131</x:v>
       </x:c>
       <x:c r="D78" s="12" t="str">
-        <x:v>Hoàng Tử Bé</x:v>
+        <x:v>Hoàng Tử Bé (Bản thường)</x:v>
       </x:c>
       <x:c r="E78" s="12" t="n">
         <x:v>1</x:v>
@@ -2791,10 +2791,10 @@
         <x:v>POS-2025-078</x:v>
       </x:c>
       <x:c r="C79" s="12" t="str">
-        <x:v>9786043950526</x:v>
+        <x:v>9786042005269</x:v>
       </x:c>
       <x:c r="D79" s="12" t="str">
-        <x:v>Spy x Family - Tập 1</x:v>
+        <x:v>Spy x Family - Tập 1 (Bản thường)</x:v>
       </x:c>
       <x:c r="E79" s="12" t="n">
         <x:v>2</x:v>
@@ -2823,10 +2823,10 @@
         <x:v>POS-2025-079</x:v>
       </x:c>
       <x:c r="C80" s="12" t="str">
-        <x:v>9786045200339</x:v>
+        <x:v>9786041200339</x:v>
       </x:c>
       <x:c r="D80" s="12" t="str">
-        <x:v>Trên Đường Băng</x:v>
+        <x:v>Trên Đường Băng (Bản thường)</x:v>
       </x:c>
       <x:c r="E80" s="12" t="n">
         <x:v>1</x:v>
@@ -2858,7 +2858,7 @@
         <x:v>9786045200261</x:v>
       </x:c>
       <x:c r="D81" s="12" t="str">
-        <x:v>Vợ Nhặt</x:v>
+        <x:v>Vợ Nhặt (Bản thường)</x:v>
       </x:c>
       <x:c r="E81" s="12" t="n">
         <x:v>2</x:v>
@@ -2890,7 +2890,7 @@
         <x:v>9786045200407</x:v>
       </x:c>
       <x:c r="D82" s="12" t="str">
-        <x:v>Nhà Giả Kim</x:v>
+        <x:v>Nhà Giả Kim (Bản thường)</x:v>
       </x:c>
       <x:c r="E82" s="12" t="n">
         <x:v>1</x:v>
@@ -2919,10 +2919,10 @@
         <x:v>POS-2025-082</x:v>
       </x:c>
       <x:c r="C83" s="12" t="str">
-        <x:v>9786045200568</x:v>
+        <x:v>9786047200568</x:v>
       </x:c>
       <x:c r="D83" s="12" t="str">
-        <x:v>Bản Đồ Cảm Xúc</x:v>
+        <x:v>Bản Đồ Cảm Xúc (Bản thường)</x:v>
       </x:c>
       <x:c r="E83" s="12" t="n">
         <x:v>1</x:v>
@@ -2954,7 +2954,7 @@
         <x:v>9786045200261</x:v>
       </x:c>
       <x:c r="D84" s="12" t="str">
-        <x:v>Vợ Nhặt</x:v>
+        <x:v>Vợ Nhặt (Bản thường)</x:v>
       </x:c>
       <x:c r="E84" s="12" t="n">
         <x:v>1</x:v>
@@ -2986,7 +2986,7 @@
         <x:v>9786045200513</x:v>
       </x:c>
       <x:c r="D85" s="12" t="str">
-        <x:v>Đọc Vị Bất Kỳ Ai</x:v>
+        <x:v>Đọc Vị Bất Kỳ Ai (Bản thường)</x:v>
       </x:c>
       <x:c r="E85" s="12" t="n">
         <x:v>1</x:v>
@@ -3018,7 +3018,7 @@
         <x:v>9786045200537</x:v>
       </x:c>
       <x:c r="D86" s="12" t="str">
-        <x:v>Tắt Đèn</x:v>
+        <x:v>Tắt Đèn (Bản thường)</x:v>
       </x:c>
       <x:c r="E86" s="12" t="n">
         <x:v>1</x:v>
@@ -3050,7 +3050,7 @@
         <x:v>9786043950410</x:v>
       </x:c>
       <x:c r="D87" s="12" t="str">
-        <x:v>Light Novel Sword Art Online 001 - Aincrad</x:v>
+        <x:v>Sword Art Online 001 - Aincrad (Bản thường)</x:v>
       </x:c>
       <x:c r="E87" s="12" t="n">
         <x:v>1</x:v>
@@ -3079,10 +3079,10 @@
         <x:v>POS-2025-087</x:v>
       </x:c>
       <x:c r="C88" s="12" t="str">
-        <x:v>9786045200568</x:v>
+        <x:v>9786047200568</x:v>
       </x:c>
       <x:c r="D88" s="12" t="str">
-        <x:v>Bản Đồ Cảm Xúc</x:v>
+        <x:v>Bản Đồ Cảm Xúc (Bản thường)</x:v>
       </x:c>
       <x:c r="E88" s="12" t="n">
         <x:v>1</x:v>
@@ -3114,7 +3114,7 @@
         <x:v>9786045200438</x:v>
       </x:c>
       <x:c r="D89" s="12" t="str">
-        <x:v>Totto-chan Bên Cửa Sổ</x:v>
+        <x:v>Totto-chan Bên Cửa Sổ (Bản thường)</x:v>
       </x:c>
       <x:c r="E89" s="12" t="n">
         <x:v>1</x:v>
@@ -3143,7 +3143,7 @@
         <x:v>POS-2025-089</x:v>
       </x:c>
       <x:c r="C90" s="12" t="str">
-        <x:v>9786043950304</x:v>
+        <x:v>9786042003045</x:v>
       </x:c>
       <x:c r="D90" s="12" t="str">
         <x:v>Dragon Ball Super - Tập 1 (Tái bản)</x:v>
@@ -3175,10 +3175,10 @@
         <x:v>POS-2025-090</x:v>
       </x:c>
       <x:c r="C91" s="12" t="str">
-        <x:v>9786043950212</x:v>
+        <x:v>9786042002121</x:v>
       </x:c>
       <x:c r="D91" s="12" t="str">
-        <x:v>One Piece - Tập 100</x:v>
+        <x:v>One Piece - Tập 100 (Bản thường)</x:v>
       </x:c>
       <x:c r="E91" s="12" t="n">
         <x:v>1</x:v>
@@ -3210,7 +3210,7 @@
         <x:v>9786045200353</x:v>
       </x:c>
       <x:c r="D92" s="12" t="str">
-        <x:v>Bài Học Diệu Kỳ Từ Cây Táo</x:v>
+        <x:v>Bài Học Diệu Kỳ Từ Cây Táo (Bản thường)</x:v>
       </x:c>
       <x:c r="E92" s="12" t="n">
         <x:v>1</x:v>
@@ -3242,7 +3242,7 @@
         <x:v>9786045200292</x:v>
       </x:c>
       <x:c r="D93" s="12" t="str">
-        <x:v>Light Novel Vì Con Gái Tôi Có Thể Đánh Bại Cả Ma Vương - Tập 1</x:v>
+        <x:v>Vì Con Gái Tôi Có Thể Đánh Bại Cả Ma Vương - Tập 1 (Bản thường)</x:v>
       </x:c>
       <x:c r="E93" s="12" t="n">
         <x:v>1</x:v>
@@ -3274,7 +3274,7 @@
         <x:v>9786045200278</x:v>
       </x:c>
       <x:c r="D94" s="12" t="str">
-        <x:v>Bố Già</x:v>
+        <x:v>Bố Già (Bản thường)</x:v>
       </x:c>
       <x:c r="E94" s="12" t="n">
         <x:v>1</x:v>
@@ -3306,7 +3306,7 @@
         <x:v>9786045200537</x:v>
       </x:c>
       <x:c r="D95" s="12" t="str">
-        <x:v>Tắt Đèn</x:v>
+        <x:v>Tắt Đèn (Bản thường)</x:v>
       </x:c>
       <x:c r="E95" s="12" t="n">
         <x:v>1</x:v>
@@ -3338,7 +3338,7 @@
         <x:v>9786045200544</x:v>
       </x:c>
       <x:c r="D96" s="12" t="str">
-        <x:v>Rừng Na Uy</x:v>
+        <x:v>Rừng Na Uy (Bản thường)</x:v>
       </x:c>
       <x:c r="E96" s="12" t="n">
         <x:v>1</x:v>
@@ -3370,7 +3370,7 @@
         <x:v>9786045200278</x:v>
       </x:c>
       <x:c r="D97" s="12" t="str">
-        <x:v>Bố Già</x:v>
+        <x:v>Bố Già (Bản thường)</x:v>
       </x:c>
       <x:c r="E97" s="12" t="n">
         <x:v>1</x:v>
@@ -3399,10 +3399,10 @@
         <x:v>POS-2025-059</x:v>
       </x:c>
       <x:c r="C98" s="12" t="str">
-        <x:v>9786045200469</x:v>
+        <x:v>9786047200469</x:v>
       </x:c>
       <x:c r="D98" s="12" t="str">
-        <x:v>Tư Duy Nhanh Và Chậm</x:v>
+        <x:v>Tư Duy Nhanh Và Chậm (Bản thường)</x:v>
       </x:c>
       <x:c r="E98" s="12" t="n">
         <x:v>1</x:v>
@@ -3431,10 +3431,10 @@
         <x:v>POS-2025-062</x:v>
       </x:c>
       <x:c r="C99" s="12" t="str">
-        <x:v>9786045200025</x:v>
+        <x:v>9786041273955</x:v>
       </x:c>
       <x:c r="D99" s="12" t="str">
-        <x:v>Tôi Thấy Hoa Vàng Trên Cỏ Xanh</x:v>
+        <x:v>Tôi Thấy Hoa Vàng Trên Cỏ Xanh (Bản thường)</x:v>
       </x:c>
       <x:c r="E99" s="12" t="n">
         <x:v>1</x:v>
@@ -3463,10 +3463,10 @@
         <x:v>POS-2025-067</x:v>
       </x:c>
       <x:c r="C100" s="12" t="str">
-        <x:v>9786043950014</x:v>
+        <x:v>9786049500141</x:v>
       </x:c>
       <x:c r="D100" s="12" t="str">
-        <x:v>Mãi Mãi Tuổi Hai Mươi (Độc quyền - Bìa cứng)</x:v>
+        <x:v>Mãi Mãi Tuổi Hai Mươi (Bản đặc biệt)</x:v>
       </x:c>
       <x:c r="E100" s="12" t="n">
         <x:v>1</x:v>
@@ -3498,7 +3498,7 @@
         <x:v>9786045200049</x:v>
       </x:c>
       <x:c r="D101" s="12" t="str">
-        <x:v>Chiếc Thuyền Ngoài Xa</x:v>
+        <x:v>Chiếc Th thuyền Ngoài Xa (Bản thường)</x:v>
       </x:c>
       <x:c r="E101" s="12" t="n">
         <x:v>1</x:v>

</xml_diff>